<commit_message>
Fix fee table empty rows and make entire row clickable
</commit_message>
<xml_diff>
--- a/backend/fees.xlsx
+++ b/backend/fees.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Shlok Parekh\Downloads\Course-Verifier-3.0\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F98051FC-85B6-4819-8300-9A6A34CAB1EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B64E2F49-30A6-4D21-A89F-C18E02B7D3E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="601" xr2:uid="{A0B92721-7CDF-495E-B956-6055A365BC29}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2493" uniqueCount="1749">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2496" uniqueCount="1752">
   <si>
     <t>Acharya Nagarjuna University</t>
   </si>
@@ -5003,10 +5003,6 @@
     <t xml:space="preserve">K S R College of Engineering (Autonomous) </t>
   </si>
   <si>
-    <t xml:space="preserve">Vidyaa Vikas College of Engineering and Technology 
-</t>
-  </si>
-  <si>
     <t xml:space="preserve">CMS College of Engineering, CMS Nagar, Eranapuram Post, Namakkal-637003. </t>
   </si>
   <si>
@@ -5022,10 +5018,6 @@
     <t xml:space="preserve">Sree Sakthi Engineering College (Autonomous), Bettathapuram, Bilichi Village </t>
   </si>
   <si>
-    <t xml:space="preserve">Coimbatore Institute of Engineering and Technology (Autonomous), Vellimalaipattinam, Narasipuram Post, 
-</t>
-  </si>
-  <si>
     <t xml:space="preserve">Dr Mahalingam College of Engineering and Technology (Autonomous) </t>
   </si>
   <si>
@@ -5297,6 +5289,21 @@
   </si>
   <si>
     <t xml:space="preserve">Indira College of Commerce and Science </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vidyaa Vikas College of Engineering and Technology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coimbatore Institute of Engineering and Technology (Autonomous), Vellimalaipattinam, Narasipuram Post, </t>
+  </si>
+  <si>
+    <t>https://admissions.psou.ac.in/asset/docs/admission/20250609105716dfabadebe8.pdf</t>
+  </si>
+  <si>
+    <t>Jagat Guru Nanak Dev Punjab State Open University</t>
+  </si>
+  <si>
+    <t>Diploma in Cyber Security</t>
   </si>
 </sst>
 </file>
@@ -5306,7 +5313,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5363,6 +5370,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -5414,7 +5428,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5481,6 +5495,8 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -6337,7 +6353,7 @@
     </row>
     <row r="28" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A28" s="11" t="s">
-        <v>1747</v>
+        <v>1745</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>46</v>
@@ -6469,7 +6485,7 @@
     </row>
     <row r="40" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A40" s="11" t="s">
-        <v>1720</v>
+        <v>1718</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>68</v>
@@ -6491,7 +6507,7 @@
     </row>
     <row r="42" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A42" s="11" t="s">
-        <v>1746</v>
+        <v>1744</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>71</v>
@@ -6524,7 +6540,7 @@
     </row>
     <row r="45" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A45" s="11" t="s">
-        <v>1745</v>
+        <v>1743</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>75</v>
@@ -6546,7 +6562,7 @@
     </row>
     <row r="47" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A47" s="11" t="s">
-        <v>1744</v>
+        <v>1742</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>79</v>
@@ -6568,7 +6584,7 @@
     </row>
     <row r="49" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A49" s="11" t="s">
-        <v>1743</v>
+        <v>1741</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>82</v>
@@ -6634,7 +6650,7 @@
     </row>
     <row r="55" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A55" s="14" t="s">
-        <v>1733</v>
+        <v>1731</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>91</v>
@@ -6920,7 +6936,7 @@
     </row>
     <row r="81" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A81" s="11" t="s">
-        <v>1748</v>
+        <v>1746</v>
       </c>
       <c r="B81" s="1" t="s">
         <v>136</v>
@@ -7030,7 +7046,7 @@
     </row>
     <row r="91" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A91" s="11" t="s">
-        <v>1692</v>
+        <v>1690</v>
       </c>
       <c r="B91" s="1" t="s">
         <v>151</v>
@@ -7173,7 +7189,7 @@
     </row>
     <row r="104" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A104" s="11" t="s">
-        <v>1691</v>
+        <v>1689</v>
       </c>
       <c r="B104" s="1" t="s">
         <v>171</v>
@@ -8900,7 +8916,7 @@
     </row>
     <row r="261" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A261" s="11" t="s">
-        <v>1734</v>
+        <v>1732</v>
       </c>
       <c r="B261" s="1" t="s">
         <v>390</v>
@@ -8911,7 +8927,7 @@
     </row>
     <row r="262" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A262" s="11" t="s">
-        <v>1735</v>
+        <v>1733</v>
       </c>
       <c r="B262" s="1" t="s">
         <v>391</v>
@@ -8922,7 +8938,7 @@
     </row>
     <row r="263" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A263" s="11" t="s">
-        <v>1736</v>
+        <v>1734</v>
       </c>
       <c r="B263" s="1" t="s">
         <v>229</v>
@@ -8933,7 +8949,7 @@
     </row>
     <row r="264" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A264" s="11" t="s">
-        <v>1737</v>
+        <v>1735</v>
       </c>
       <c r="B264" s="1" t="s">
         <v>229</v>
@@ -8944,7 +8960,7 @@
     </row>
     <row r="265" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A265" s="11" t="s">
-        <v>1738</v>
+        <v>1736</v>
       </c>
       <c r="B265" s="1" t="s">
         <v>229</v>
@@ -8955,7 +8971,7 @@
     </row>
     <row r="266" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A266" s="11" t="s">
-        <v>1739</v>
+        <v>1737</v>
       </c>
       <c r="B266" s="1" t="s">
         <v>229</v>
@@ -8966,7 +8982,7 @@
     </row>
     <row r="267" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A267" s="11" t="s">
-        <v>1740</v>
+        <v>1738</v>
       </c>
       <c r="B267" s="1" t="s">
         <v>390</v>
@@ -8977,7 +8993,7 @@
     </row>
     <row r="268" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A268" s="11" t="s">
-        <v>1741</v>
+        <v>1739</v>
       </c>
       <c r="B268" s="1" t="s">
         <v>390</v>
@@ -8988,7 +9004,7 @@
     </row>
     <row r="269" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A269" s="11" t="s">
-        <v>1742</v>
+        <v>1740</v>
       </c>
       <c r="B269" s="1" t="s">
         <v>229</v>
@@ -9109,7 +9125,7 @@
     </row>
     <row r="280" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A280" s="11" t="s">
-        <v>1721</v>
+        <v>1719</v>
       </c>
       <c r="B280" s="1" t="s">
         <v>150</v>
@@ -9120,7 +9136,7 @@
     </row>
     <row r="281" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A281" s="11" t="s">
-        <v>1722</v>
+        <v>1720</v>
       </c>
       <c r="B281" s="1" t="s">
         <v>403</v>
@@ -9175,7 +9191,7 @@
     </row>
     <row r="286" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A286" s="11" t="s">
-        <v>1723</v>
+        <v>1721</v>
       </c>
       <c r="B286" s="1" t="s">
         <v>390</v>
@@ -9197,7 +9213,7 @@
     </row>
     <row r="288" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A288" s="11" t="s">
-        <v>1724</v>
+        <v>1722</v>
       </c>
       <c r="B288" s="1" t="s">
         <v>390</v>
@@ -9208,7 +9224,7 @@
     </row>
     <row r="289" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A289" s="11" t="s">
-        <v>1725</v>
+        <v>1723</v>
       </c>
       <c r="B289" s="1" t="s">
         <v>406</v>
@@ -9219,7 +9235,7 @@
     </row>
     <row r="290" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A290" s="11" t="s">
-        <v>1726</v>
+        <v>1724</v>
       </c>
       <c r="B290" s="1" t="s">
         <v>390</v>
@@ -9230,7 +9246,7 @@
     </row>
     <row r="291" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A291" s="11" t="s">
-        <v>1727</v>
+        <v>1725</v>
       </c>
       <c r="B291" s="1" t="s">
         <v>202</v>
@@ -9241,7 +9257,7 @@
     </row>
     <row r="292" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A292" s="11" t="s">
-        <v>1728</v>
+        <v>1726</v>
       </c>
       <c r="B292" s="1" t="s">
         <v>390</v>
@@ -9263,7 +9279,7 @@
     </row>
     <row r="294" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A294" s="11" t="s">
-        <v>1722</v>
+        <v>1720</v>
       </c>
       <c r="B294" s="1" t="s">
         <v>408</v>
@@ -9692,7 +9708,7 @@
     </row>
     <row r="333" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A333" s="11" t="s">
-        <v>1703</v>
+        <v>1701</v>
       </c>
       <c r="B333" s="1" t="s">
         <v>30</v>
@@ -9714,7 +9730,7 @@
     </row>
     <row r="335" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A335" s="11" t="s">
-        <v>1704</v>
+        <v>1702</v>
       </c>
       <c r="B335" s="1" t="s">
         <v>30</v>
@@ -9725,7 +9741,7 @@
     </row>
     <row r="336" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A336" s="11" t="s">
-        <v>1705</v>
+        <v>1703</v>
       </c>
       <c r="B336" s="1" t="s">
         <v>421</v>
@@ -9736,7 +9752,7 @@
     </row>
     <row r="337" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A337" s="11" t="s">
-        <v>1706</v>
+        <v>1704</v>
       </c>
       <c r="B337" s="1" t="s">
         <v>422</v>
@@ -9747,7 +9763,7 @@
     </row>
     <row r="338" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A338" s="11" t="s">
-        <v>1707</v>
+        <v>1705</v>
       </c>
       <c r="B338" s="1" t="s">
         <v>30</v>
@@ -9758,7 +9774,7 @@
     </row>
     <row r="339" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A339" s="11" t="s">
-        <v>1708</v>
+        <v>1706</v>
       </c>
       <c r="B339" s="1" t="s">
         <v>30</v>
@@ -9769,7 +9785,7 @@
     </row>
     <row r="340" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A340" s="11" t="s">
-        <v>1709</v>
+        <v>1707</v>
       </c>
       <c r="B340" s="1" t="s">
         <v>30</v>
@@ -9835,7 +9851,7 @@
     </row>
     <row r="346" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A346" s="11" t="s">
-        <v>1710</v>
+        <v>1708</v>
       </c>
       <c r="B346" s="1" t="s">
         <v>30</v>
@@ -9846,7 +9862,7 @@
     </row>
     <row r="347" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A347" s="11" t="s">
-        <v>1711</v>
+        <v>1709</v>
       </c>
       <c r="B347" s="1" t="s">
         <v>30</v>
@@ -9857,7 +9873,7 @@
     </row>
     <row r="348" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A348" s="11" t="s">
-        <v>1712</v>
+        <v>1710</v>
       </c>
       <c r="B348" s="1" t="s">
         <v>30</v>
@@ -9868,7 +9884,7 @@
     </row>
     <row r="349" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A349" s="11" t="s">
-        <v>1713</v>
+        <v>1711</v>
       </c>
       <c r="B349" s="1" t="s">
         <v>30</v>
@@ -9879,7 +9895,7 @@
     </row>
     <row r="350" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A350" s="11" t="s">
-        <v>1714</v>
+        <v>1712</v>
       </c>
       <c r="B350" s="1" t="s">
         <v>30</v>
@@ -9890,7 +9906,7 @@
     </row>
     <row r="351" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A351" s="11" t="s">
-        <v>1715</v>
+        <v>1713</v>
       </c>
       <c r="B351" s="1" t="s">
         <v>30</v>
@@ -9901,7 +9917,7 @@
     </row>
     <row r="352" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A352" s="11" t="s">
-        <v>1716</v>
+        <v>1714</v>
       </c>
       <c r="B352" s="1" t="s">
         <v>30</v>
@@ -9987,7 +10003,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="360" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:3" ht="28.5" x14ac:dyDescent="0.35">
       <c r="A360" s="14" t="s">
         <v>1611</v>
       </c>
@@ -10055,7 +10071,7 @@
     </row>
     <row r="366" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A366" s="11" t="s">
-        <v>1729</v>
+        <v>1727</v>
       </c>
       <c r="B366" s="1" t="s">
         <v>424</v>
@@ -10264,7 +10280,7 @@
     </row>
     <row r="385" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A385" s="11" t="s">
-        <v>1730</v>
+        <v>1728</v>
       </c>
       <c r="B385" s="1" t="s">
         <v>430</v>
@@ -10473,7 +10489,7 @@
     </row>
     <row r="404" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A404" s="14" t="s">
-        <v>1702</v>
+        <v>1700</v>
       </c>
       <c r="B404" s="1" t="s">
         <v>433</v>
@@ -10572,7 +10588,7 @@
     </row>
     <row r="413" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A413" s="11" t="s">
-        <v>1717</v>
+        <v>1715</v>
       </c>
       <c r="B413" s="1" t="s">
         <v>319</v>
@@ -10583,7 +10599,7 @@
     </row>
     <row r="414" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A414" s="11" t="s">
-        <v>1718</v>
+        <v>1716</v>
       </c>
       <c r="B414" s="1" t="s">
         <v>442</v>
@@ -10594,7 +10610,7 @@
     </row>
     <row r="415" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A415" s="11" t="s">
-        <v>1719</v>
+        <v>1717</v>
       </c>
       <c r="B415" s="1" t="s">
         <v>299</v>
@@ -10737,7 +10753,7 @@
     </row>
     <row r="428" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A428" s="11" t="s">
-        <v>1693</v>
+        <v>1691</v>
       </c>
       <c r="B428" s="1" t="s">
         <v>454</v>
@@ -10748,7 +10764,7 @@
     </row>
     <row r="429" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A429" s="11" t="s">
-        <v>1694</v>
+        <v>1692</v>
       </c>
       <c r="B429" s="1" t="s">
         <v>320</v>
@@ -10781,7 +10797,7 @@
     </row>
     <row r="432" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A432" s="11" t="s">
-        <v>1695</v>
+        <v>1693</v>
       </c>
       <c r="B432" s="1" t="s">
         <v>458</v>
@@ -10792,7 +10808,7 @@
     </row>
     <row r="433" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A433" s="11" t="s">
-        <v>1696</v>
+        <v>1694</v>
       </c>
       <c r="B433" s="1" t="s">
         <v>459</v>
@@ -10814,7 +10830,7 @@
     </row>
     <row r="435" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A435" s="11" t="s">
-        <v>1697</v>
+        <v>1695</v>
       </c>
       <c r="B435" s="1" t="s">
         <v>459</v>
@@ -10825,7 +10841,7 @@
     </row>
     <row r="436" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A436" s="11" t="s">
-        <v>1698</v>
+        <v>1696</v>
       </c>
       <c r="B436" s="1" t="s">
         <v>459</v>
@@ -10836,7 +10852,7 @@
     </row>
     <row r="437" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A437" s="11" t="s">
-        <v>1699</v>
+        <v>1697</v>
       </c>
       <c r="B437" s="1" t="s">
         <v>459</v>
@@ -10847,7 +10863,7 @@
     </row>
     <row r="438" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A438" s="11" t="s">
-        <v>1699</v>
+        <v>1697</v>
       </c>
       <c r="B438" s="1" t="s">
         <v>454</v>
@@ -10858,7 +10874,7 @@
     </row>
     <row r="439" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A439" s="11" t="s">
-        <v>1700</v>
+        <v>1698</v>
       </c>
       <c r="B439" s="1" t="s">
         <v>462</v>
@@ -10869,7 +10885,7 @@
     </row>
     <row r="440" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A440" s="11" t="s">
-        <v>1701</v>
+        <v>1699</v>
       </c>
       <c r="B440" s="1" t="s">
         <v>463</v>
@@ -10880,7 +10896,7 @@
     </row>
     <row r="441" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A441" s="11" t="s">
-        <v>1731</v>
+        <v>1729</v>
       </c>
       <c r="B441" s="1" t="s">
         <v>464</v>
@@ -10891,7 +10907,7 @@
     </row>
     <row r="442" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A442" s="11" t="s">
-        <v>1732</v>
+        <v>1730</v>
       </c>
       <c r="B442" s="1" t="s">
         <v>430</v>
@@ -10902,7 +10918,7 @@
     </row>
     <row r="443" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A443" s="14" t="s">
-        <v>1651</v>
+        <v>1747</v>
       </c>
       <c r="B443" s="1" t="s">
         <v>465</v>
@@ -10913,7 +10929,7 @@
     </row>
     <row r="444" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A444" s="11" t="s">
-        <v>1652</v>
+        <v>1651</v>
       </c>
       <c r="B444" s="1" t="s">
         <v>465</v>
@@ -10924,7 +10940,7 @@
     </row>
     <row r="445" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A445" s="11" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="B445" s="1" t="s">
         <v>465</v>
@@ -10935,7 +10951,7 @@
     </row>
     <row r="446" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A446" s="11" t="s">
-        <v>1654</v>
+        <v>1653</v>
       </c>
       <c r="B446" s="1" t="s">
         <v>465</v>
@@ -10946,7 +10962,7 @@
     </row>
     <row r="447" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A447" s="11" t="s">
-        <v>1655</v>
+        <v>1654</v>
       </c>
       <c r="B447" s="1" t="s">
         <v>465</v>
@@ -10957,7 +10973,7 @@
     </row>
     <row r="448" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A448" s="11" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="B448" s="1" t="s">
         <v>465</v>
@@ -10968,7 +10984,7 @@
     </row>
     <row r="449" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A449" s="14" t="s">
-        <v>1657</v>
+        <v>1748</v>
       </c>
       <c r="B449" s="1" t="s">
         <v>465</v>
@@ -10979,7 +10995,7 @@
     </row>
     <row r="450" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A450" s="11" t="s">
-        <v>1658</v>
+        <v>1656</v>
       </c>
       <c r="B450" s="1" t="s">
         <v>465</v>
@@ -10990,7 +11006,7 @@
     </row>
     <row r="451" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A451" s="11" t="s">
-        <v>1659</v>
+        <v>1657</v>
       </c>
       <c r="B451" s="1" t="s">
         <v>465</v>
@@ -11001,7 +11017,7 @@
     </row>
     <row r="452" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A452" s="11" t="s">
-        <v>1660</v>
+        <v>1658</v>
       </c>
       <c r="B452" s="1" t="s">
         <v>465</v>
@@ -11012,7 +11028,7 @@
     </row>
     <row r="453" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A453" s="11" t="s">
-        <v>1661</v>
+        <v>1659</v>
       </c>
       <c r="B453" s="1" t="s">
         <v>465</v>
@@ -11023,7 +11039,7 @@
     </row>
     <row r="454" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A454" s="11" t="s">
-        <v>1662</v>
+        <v>1660</v>
       </c>
       <c r="B454" s="1" t="s">
         <v>465</v>
@@ -11045,7 +11061,7 @@
     </row>
     <row r="456" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A456" s="11" t="s">
-        <v>1663</v>
+        <v>1661</v>
       </c>
       <c r="B456" s="1" t="s">
         <v>465</v>
@@ -11056,7 +11072,7 @@
     </row>
     <row r="457" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A457" s="11" t="s">
-        <v>1664</v>
+        <v>1662</v>
       </c>
       <c r="B457" s="1" t="s">
         <v>465</v>
@@ -11067,7 +11083,7 @@
     </row>
     <row r="458" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A458" s="11" t="s">
-        <v>1665</v>
+        <v>1663</v>
       </c>
       <c r="B458" s="1" t="s">
         <v>465</v>
@@ -11078,7 +11094,7 @@
     </row>
     <row r="459" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A459" s="11" t="s">
-        <v>1666</v>
+        <v>1664</v>
       </c>
       <c r="B459" s="1" t="s">
         <v>465</v>
@@ -11089,7 +11105,7 @@
     </row>
     <row r="460" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A460" s="11" t="s">
-        <v>1667</v>
+        <v>1665</v>
       </c>
       <c r="B460" s="1" t="s">
         <v>465</v>
@@ -11100,7 +11116,7 @@
     </row>
     <row r="461" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A461" s="11" t="s">
-        <v>1668</v>
+        <v>1666</v>
       </c>
       <c r="B461" s="1" t="s">
         <v>465</v>
@@ -11111,7 +11127,7 @@
     </row>
     <row r="462" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A462" s="11" t="s">
-        <v>1669</v>
+        <v>1667</v>
       </c>
       <c r="B462" s="1" t="s">
         <v>465</v>
@@ -11122,7 +11138,7 @@
     </row>
     <row r="463" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A463" s="11" t="s">
-        <v>1670</v>
+        <v>1668</v>
       </c>
       <c r="B463" s="1" t="s">
         <v>465</v>
@@ -11133,7 +11149,7 @@
     </row>
     <row r="464" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A464" s="11" t="s">
-        <v>1671</v>
+        <v>1669</v>
       </c>
       <c r="B464" s="1" t="s">
         <v>465</v>
@@ -11144,7 +11160,7 @@
     </row>
     <row r="465" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A465" s="11" t="s">
-        <v>1672</v>
+        <v>1670</v>
       </c>
       <c r="B465" s="1" t="s">
         <v>465</v>
@@ -11155,7 +11171,7 @@
     </row>
     <row r="466" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A466" s="11" t="s">
-        <v>1673</v>
+        <v>1671</v>
       </c>
       <c r="B466" s="1" t="s">
         <v>465</v>
@@ -11166,7 +11182,7 @@
     </row>
     <row r="467" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A467" s="11" t="s">
-        <v>1674</v>
+        <v>1672</v>
       </c>
       <c r="B467" s="1" t="s">
         <v>465</v>
@@ -11177,7 +11193,7 @@
     </row>
     <row r="468" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A468" s="11" t="s">
-        <v>1675</v>
+        <v>1673</v>
       </c>
       <c r="B468" s="1" t="s">
         <v>465</v>
@@ -11188,7 +11204,7 @@
     </row>
     <row r="469" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A469" s="11" t="s">
-        <v>1676</v>
+        <v>1674</v>
       </c>
       <c r="B469" s="1" t="s">
         <v>465</v>
@@ -11199,7 +11215,7 @@
     </row>
     <row r="470" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A470" s="11" t="s">
-        <v>1677</v>
+        <v>1675</v>
       </c>
       <c r="B470" s="1" t="s">
         <v>465</v>
@@ -11210,7 +11226,7 @@
     </row>
     <row r="471" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A471" s="11" t="s">
-        <v>1678</v>
+        <v>1676</v>
       </c>
       <c r="B471" s="1" t="s">
         <v>465</v>
@@ -11221,7 +11237,7 @@
     </row>
     <row r="472" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A472" s="11" t="s">
-        <v>1679</v>
+        <v>1677</v>
       </c>
       <c r="B472" s="1" t="s">
         <v>465</v>
@@ -11232,7 +11248,7 @@
     </row>
     <row r="473" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A473" s="11" t="s">
-        <v>1680</v>
+        <v>1678</v>
       </c>
       <c r="B473" s="1" t="s">
         <v>465</v>
@@ -11243,7 +11259,7 @@
     </row>
     <row r="474" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A474" s="11" t="s">
-        <v>1681</v>
+        <v>1679</v>
       </c>
       <c r="B474" s="1" t="s">
         <v>465</v>
@@ -11254,7 +11270,7 @@
     </row>
     <row r="475" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A475" s="11" t="s">
-        <v>1682</v>
+        <v>1680</v>
       </c>
       <c r="B475" s="1" t="s">
         <v>465</v>
@@ -11265,7 +11281,7 @@
     </row>
     <row r="476" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A476" s="11" t="s">
-        <v>1683</v>
+        <v>1681</v>
       </c>
       <c r="B476" s="1" t="s">
         <v>465</v>
@@ -11276,7 +11292,7 @@
     </row>
     <row r="477" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A477" s="11" t="s">
-        <v>1684</v>
+        <v>1682</v>
       </c>
       <c r="B477" s="1" t="s">
         <v>465</v>
@@ -11287,7 +11303,7 @@
     </row>
     <row r="478" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A478" s="11" t="s">
-        <v>1685</v>
+        <v>1683</v>
       </c>
       <c r="B478" s="1" t="s">
         <v>465</v>
@@ -11298,7 +11314,7 @@
     </row>
     <row r="479" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A479" s="11" t="s">
-        <v>1686</v>
+        <v>1684</v>
       </c>
       <c r="B479" s="1" t="s">
         <v>465</v>
@@ -11309,7 +11325,7 @@
     </row>
     <row r="480" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A480" s="11" t="s">
-        <v>1687</v>
+        <v>1685</v>
       </c>
       <c r="B480" s="1" t="s">
         <v>465</v>
@@ -11320,7 +11336,7 @@
     </row>
     <row r="481" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A481" s="11" t="s">
-        <v>1688</v>
+        <v>1686</v>
       </c>
       <c r="B481" s="1" t="s">
         <v>465</v>
@@ -11331,7 +11347,7 @@
     </row>
     <row r="482" spans="1:3" s="19" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A482" s="11" t="s">
-        <v>1689</v>
+        <v>1687</v>
       </c>
       <c r="B482" s="1" t="s">
         <v>465</v>
@@ -11353,7 +11369,7 @@
     </row>
     <row r="484" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A484" s="11" t="s">
-        <v>1690</v>
+        <v>1688</v>
       </c>
       <c r="B484" s="1" t="s">
         <v>465</v>
@@ -15168,19 +15184,27 @@
         <v>1580</v>
       </c>
     </row>
-    <row r="831" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A831" t="s">
+    <row r="831" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A831" s="30" t="s">
         <v>1592</v>
       </c>
       <c r="B831" s="1" t="s">
         <v>1594</v>
       </c>
-      <c r="C831" s="12" t="s">
+      <c r="C831" s="31" t="s">
         <v>1593</v>
       </c>
     </row>
-    <row r="832" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C832" s="21"/>
+    <row r="832" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A832" s="1" t="s">
+        <v>1750</v>
+      </c>
+      <c r="B832" s="1" t="s">
+        <v>1751</v>
+      </c>
+      <c r="C832" s="12" t="s">
+        <v>1749</v>
+      </c>
     </row>
     <row r="833" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C833" s="21"/>
@@ -20495,11 +20519,12 @@
     <hyperlink ref="C829" r:id="rId695" xr:uid="{8D5E4FFD-4295-40FC-80CE-939CE9A373E4}"/>
     <hyperlink ref="C830" r:id="rId696" xr:uid="{3948E6EA-1427-48E4-8A29-41429A28459B}"/>
     <hyperlink ref="C831" r:id="rId697" xr:uid="{C6DDC614-32F2-47BD-BE28-A0DA73586335}"/>
+    <hyperlink ref="C832" r:id="rId698" xr:uid="{19E7F49A-95CD-4A49-A16A-191D7E976B13}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId698"/>
+  <pageSetup orientation="portrait" r:id="rId699"/>
   <tableParts count="1">
-    <tablePart r:id="rId699"/>
+    <tablePart r:id="rId700"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>